<commit_message>
Sync workshop test data from source of truth
Refresh the served datasets to match female-health/landing (the source
of truth). The live workshop was serving a pre-strengthening dataset.

- cycle_test_data.csv: ovulation signals now in most cycles
  (high energy 3 -> 13 days, added "increased libido"); 91 -> 109 rows
- wearable_test_data.csv: deeper luteal HRV dip (follicular-high ->
  luteal-low -> pre-period crash)
- merged_test_data.csv + .xlsx: regenerated answer key to match
- index.html: update FILE 1 download-card label (91 rows, 2 KB ->
  109 rows, 3 KB); wearable card unchanged (still 176 rows, 5 KB)

Page structure, prompts and expected-result descriptions unchanged.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012wFqHjHyYrz8x44QT9Sbrq
</commit_message>
<xml_diff>
--- a/merged_test_data.xlsx
+++ b/merged_test_data.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="merged" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="merged" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -759,16 +759,16 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>8.1</v>
+        <v>7.4</v>
       </c>
       <c r="F13" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G13" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H13" t="n">
-        <v>36.1</v>
+        <v>36.13</v>
       </c>
     </row>
     <row r="14">
@@ -777,17 +777,22 @@
           <t>2026-01-13</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>great</t>
+        </is>
+      </c>
       <c r="E14" t="n">
-        <v>7.5</v>
+        <v>7.1</v>
       </c>
       <c r="F14" t="n">
         <v>57</v>
       </c>
       <c r="G14" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="H14" t="n">
-        <v>36.15</v>
+        <v>36.26</v>
       </c>
     </row>
     <row r="15">
@@ -796,17 +801,22 @@
           <t>2026-01-14</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E15" t="n">
-        <v>7.3</v>
+        <v>6.8</v>
       </c>
       <c r="F15" t="n">
         <v>57</v>
       </c>
       <c r="G15" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H15" t="n">
-        <v>36.19</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="16">
@@ -816,16 +826,16 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="F16" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G16" t="n">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="H16" t="n">
-        <v>36.35</v>
+        <v>36.34</v>
       </c>
     </row>
     <row r="17">
@@ -835,16 +845,16 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>6.9</v>
+        <v>7</v>
       </c>
       <c r="F17" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G17" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="H17" t="n">
-        <v>36.47</v>
+        <v>36.53</v>
       </c>
     </row>
     <row r="18">
@@ -853,17 +863,22 @@
           <t>2026-01-17</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E18" t="n">
-        <v>7.4</v>
+        <v>7</v>
       </c>
       <c r="F18" t="n">
         <v>61</v>
       </c>
       <c r="G18" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H18" t="n">
-        <v>36.55</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="19">
@@ -872,14 +887,19 @@
           <t>2026-01-18</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E19" t="n">
-        <v>7.6</v>
+        <v>7.3</v>
       </c>
       <c r="F19" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G19" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H19" t="n">
         <v>36.55</v>
@@ -893,20 +913,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>7.8</v>
+        <v>7.2</v>
       </c>
       <c r="F20" t="n">
         <v>60</v>
       </c>
       <c r="G20" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H20" t="n">
-        <v>36.39</v>
+        <v>36.43</v>
       </c>
     </row>
     <row r="21">
@@ -915,17 +935,22 @@
           <t>2026-01-20</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E21" t="n">
-        <v>6.9</v>
+        <v>6.4</v>
       </c>
       <c r="F21" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G21" t="n">
         <v>58</v>
       </c>
       <c r="H21" t="n">
-        <v>36.5</v>
+        <v>36.47</v>
       </c>
     </row>
     <row r="22">
@@ -935,16 +960,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>7.3</v>
+        <v>6.9</v>
       </c>
       <c r="F22" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G22" t="n">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="H22" t="n">
-        <v>36.42</v>
+        <v>36.52</v>
       </c>
     </row>
     <row r="23">
@@ -953,22 +978,17 @@
           <t>2026-01-22</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="E23" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="F23" t="n">
+        <v>62</v>
+      </c>
+      <c r="G23" t="n">
         <v>63</v>
       </c>
-      <c r="G23" t="n">
-        <v>67</v>
-      </c>
       <c r="H23" t="n">
-        <v>36.51</v>
+        <v>36.56</v>
       </c>
     </row>
     <row r="24">
@@ -977,22 +997,17 @@
           <t>2026-01-23</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="E24" t="n">
-        <v>6.5</v>
+        <v>7.4</v>
       </c>
       <c r="F24" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G24" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H24" t="n">
-        <v>36.44</v>
+        <v>36.42</v>
       </c>
     </row>
     <row r="25">
@@ -1003,7 +1018,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>poor sleep</t>
+          <t>bloating</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1012,16 +1027,16 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>8.1</v>
+        <v>6.7</v>
       </c>
       <c r="F25" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G25" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H25" t="n">
-        <v>36.55</v>
+        <v>36.58</v>
       </c>
     </row>
     <row r="26">
@@ -1030,27 +1045,17 @@
           <t>2026-01-25</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>bloating</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>okay</t>
-        </is>
-      </c>
       <c r="E26" t="n">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="F26" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G26" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H26" t="n">
-        <v>36.47</v>
+        <v>36.48</v>
       </c>
     </row>
     <row r="27">
@@ -1061,25 +1066,25 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>sore breasts</t>
+          <t>headache</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="F27" t="n">
         <v>62</v>
       </c>
       <c r="G27" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="H27" t="n">
-        <v>36.39</v>
+        <v>36.53</v>
       </c>
     </row>
     <row r="28">
@@ -1088,17 +1093,22 @@
           <t>2026-01-27</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
       <c r="E28" t="n">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="F28" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G28" t="n">
         <v>48</v>
       </c>
       <c r="H28" t="n">
-        <v>36.33</v>
+        <v>36.28</v>
       </c>
     </row>
     <row r="29">
@@ -1107,13 +1117,18 @@
           <t>2026-01-28</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>bloating</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="F29" t="n">
         <v>62</v>
@@ -1122,7 +1137,7 @@
         <v>45</v>
       </c>
       <c r="H29" t="n">
-        <v>36.29</v>
+        <v>36.31</v>
       </c>
     </row>
     <row r="30">
@@ -1147,16 +1162,16 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>8.199999999999999</v>
+        <v>7.1</v>
       </c>
       <c r="F30" t="n">
         <v>57</v>
       </c>
       <c r="G30" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H30" t="n">
-        <v>36.22</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="31">
@@ -1170,22 +1185,27 @@
           <t>heavy</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>backache</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>7.9</v>
+        <v>7.7</v>
       </c>
       <c r="F31" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G31" t="n">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="H31" t="n">
-        <v>36.13</v>
+        <v>36.16</v>
       </c>
     </row>
     <row r="32">
@@ -1205,16 +1225,16 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>7.7</v>
+        <v>7.6</v>
       </c>
       <c r="F32" t="n">
         <v>58</v>
       </c>
       <c r="G32" t="n">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="H32" t="n">
-        <v>36.16</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="33">
@@ -1234,13 +1254,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>7.6</v>
+        <v>7.4</v>
       </c>
       <c r="F33" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G33" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="H33" t="n">
         <v>36.18</v>
@@ -1263,16 +1283,16 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="F34" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G34" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H34" t="n">
-        <v>36.18</v>
+        <v>36.06</v>
       </c>
     </row>
     <row r="35">
@@ -1282,16 +1302,16 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="F35" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G35" t="n">
         <v>69</v>
       </c>
       <c r="H35" t="n">
-        <v>36.06</v>
+        <v>36.1</v>
       </c>
     </row>
     <row r="36">
@@ -1300,17 +1320,22 @@
           <t>2026-02-04</t>
         </is>
       </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E36" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="F36" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G36" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="H36" t="n">
-        <v>36.1</v>
+        <v>36.15</v>
       </c>
     </row>
     <row r="37">
@@ -1325,13 +1350,13 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="F37" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G37" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H37" t="n">
         <v>36.15</v>
@@ -1343,22 +1368,17 @@
           <t>2026-02-06</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>okay</t>
-        </is>
-      </c>
       <c r="E38" t="n">
-        <v>7.5</v>
+        <v>7.6</v>
       </c>
       <c r="F38" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G38" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H38" t="n">
-        <v>36.15</v>
+        <v>36.17</v>
       </c>
     </row>
     <row r="39">
@@ -1367,17 +1387,22 @@
           <t>2026-02-07</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E39" t="n">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="F39" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G39" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H39" t="n">
-        <v>36.17</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="40">
@@ -1386,22 +1411,17 @@
           <t>2026-02-08</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>okay</t>
-        </is>
-      </c>
       <c r="E40" t="n">
         <v>7.5</v>
       </c>
       <c r="F40" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G40" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H40" t="n">
-        <v>36.18</v>
+        <v>36.15</v>
       </c>
     </row>
     <row r="41">
@@ -1410,17 +1430,22 @@
           <t>2026-02-09</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E41" t="n">
-        <v>7.5</v>
+        <v>7.1</v>
       </c>
       <c r="F41" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G41" t="n">
         <v>70</v>
       </c>
       <c r="H41" t="n">
-        <v>36.15</v>
+        <v>36.02</v>
       </c>
     </row>
     <row r="42">
@@ -1429,9 +1454,14 @@
           <t>2026-02-10</t>
         </is>
       </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>high energy</t>
+        </is>
+      </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
     </row>
@@ -1441,17 +1471,27 @@
           <t>2026-02-11</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>high energy</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>great</t>
+        </is>
+      </c>
       <c r="E43" t="n">
-        <v>7.1</v>
+        <v>7.4</v>
       </c>
       <c r="F43" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G43" t="n">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H43" t="n">
-        <v>36.24</v>
+        <v>36.15</v>
       </c>
     </row>
     <row r="44">
@@ -1460,22 +1500,27 @@
           <t>2026-02-12</t>
         </is>
       </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>high energy</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>great</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>7.4</v>
+        <v>7.8</v>
       </c>
       <c r="F44" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G44" t="n">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="H44" t="n">
-        <v>36.2</v>
+        <v>36.22</v>
       </c>
     </row>
     <row r="45">
@@ -1484,27 +1529,22 @@
           <t>2026-02-13</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>high energy</t>
-        </is>
-      </c>
       <c r="D45" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="F45" t="n">
         <v>58</v>
       </c>
       <c r="G45" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="H45" t="n">
-        <v>36.4</v>
+        <v>36.27</v>
       </c>
     </row>
     <row r="46">
@@ -1513,17 +1553,22 @@
           <t>2026-02-14</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E46" t="n">
-        <v>7.8</v>
+        <v>7.5</v>
       </c>
       <c r="F46" t="n">
+        <v>61</v>
+      </c>
+      <c r="G46" t="n">
         <v>58</v>
       </c>
-      <c r="G46" t="n">
-        <v>59</v>
-      </c>
       <c r="H46" t="n">
-        <v>36.42</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="47">
@@ -1532,22 +1577,17 @@
           <t>2026-02-15</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="E47" t="n">
-        <v>7.9</v>
+        <v>7.5</v>
       </c>
       <c r="F47" t="n">
         <v>61</v>
       </c>
       <c r="G47" t="n">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="H47" t="n">
-        <v>36.49</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="48">
@@ -1556,22 +1596,17 @@
           <t>2026-02-16</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>okay</t>
-        </is>
-      </c>
       <c r="E48" t="n">
-        <v>6.8</v>
+        <v>7.1</v>
       </c>
       <c r="F48" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G48" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="H48" t="n">
-        <v>36.54</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="49">
@@ -1581,16 +1616,16 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>7.9</v>
+        <v>6.9</v>
       </c>
       <c r="F49" t="n">
+        <v>61</v>
+      </c>
+      <c r="G49" t="n">
         <v>62</v>
       </c>
-      <c r="G49" t="n">
-        <v>56</v>
-      </c>
       <c r="H49" t="n">
-        <v>36.53</v>
+        <v>36.43</v>
       </c>
     </row>
     <row r="50">
@@ -1599,8 +1634,13 @@
           <t>2026-02-18</t>
         </is>
       </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E50" t="n">
-        <v>6.9</v>
+        <v>7.3</v>
       </c>
       <c r="F50" t="n">
         <v>61</v>
@@ -1609,7 +1649,7 @@
         <v>59</v>
       </c>
       <c r="H50" t="n">
-        <v>36.5</v>
+        <v>36.45</v>
       </c>
     </row>
     <row r="51">
@@ -1618,14 +1658,19 @@
           <t>2026-02-19</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E51" t="n">
-        <v>7.5</v>
+        <v>6.8</v>
       </c>
       <c r="F51" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G51" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="H51" t="n">
         <v>36.51</v>
@@ -1638,16 +1683,16 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
       <c r="F52" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G52" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H52" t="n">
-        <v>36.54</v>
+        <v>36.42</v>
       </c>
     </row>
     <row r="53">
@@ -1656,17 +1701,22 @@
           <t>2026-02-21</t>
         </is>
       </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E53" t="n">
-        <v>7.8</v>
+        <v>7.4</v>
       </c>
       <c r="F53" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G53" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="H53" t="n">
-        <v>36.54</v>
+        <v>36.53</v>
       </c>
     </row>
     <row r="54">
@@ -1676,16 +1726,16 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>7.5</v>
+        <v>7.3</v>
       </c>
       <c r="F54" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G54" t="n">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="H54" t="n">
-        <v>36.47</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="55">
@@ -1694,27 +1744,17 @@
           <t>2026-02-23</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>cravings</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
       <c r="E55" t="n">
-        <v>7.3</v>
+        <v>7</v>
       </c>
       <c r="F55" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G55" t="n">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="H55" t="n">
-        <v>36.54</v>
+        <v>36.41</v>
       </c>
     </row>
     <row r="56">
@@ -1725,25 +1765,25 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>sore breasts</t>
+          <t>cravings</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>irritable</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>6.2</v>
+        <v>6.4</v>
       </c>
       <c r="F56" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G56" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="H56" t="n">
-        <v>36.51</v>
+        <v>36.56</v>
       </c>
     </row>
     <row r="57">
@@ -1752,27 +1792,17 @@
           <t>2026-02-25</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>headache</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>irritable</t>
-        </is>
-      </c>
       <c r="E57" t="n">
-        <v>6.6</v>
+        <v>7.1</v>
       </c>
       <c r="F57" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G57" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="H57" t="n">
-        <v>36.34</v>
+        <v>36.29</v>
       </c>
     </row>
     <row r="58">
@@ -1783,25 +1813,25 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>headache</t>
+          <t>bloating</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>6.8</v>
+        <v>6.2</v>
       </c>
       <c r="F58" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G58" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="H58" t="n">
-        <v>36.33</v>
+        <v>36.34</v>
       </c>
     </row>
     <row r="59">
@@ -1815,22 +1845,27 @@
           <t>heavy</t>
         </is>
       </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>backache</t>
+        </is>
+      </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>7.4</v>
+        <v>7.8</v>
       </c>
       <c r="F59" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G59" t="n">
         <v>65</v>
       </c>
       <c r="H59" t="n">
-        <v>36.14</v>
+        <v>36.08</v>
       </c>
     </row>
     <row r="60">
@@ -1844,22 +1879,27 @@
           <t>heavy</t>
         </is>
       </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>backache</t>
+        </is>
+      </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>8.1</v>
+        <v>7.2</v>
       </c>
       <c r="F60" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G60" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H60" t="n">
-        <v>36.04</v>
+        <v>36.21</v>
       </c>
     </row>
     <row r="61">
@@ -1875,25 +1915,25 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>low energy</t>
+          <t>headache</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>7.7</v>
+        <v>7.3</v>
       </c>
       <c r="F61" t="n">
         <v>57</v>
       </c>
       <c r="G61" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="H61" t="n">
-        <v>36.17</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="62">
@@ -1909,20 +1949,20 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>7.2</v>
+        <v>6.8</v>
       </c>
       <c r="F62" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G62" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="H62" t="n">
-        <v>36.13</v>
+        <v>36.07</v>
       </c>
     </row>
     <row r="63">
@@ -1942,16 +1982,16 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>6.8</v>
+        <v>7.3</v>
       </c>
       <c r="F63" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G63" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H63" t="n">
-        <v>36.05</v>
+        <v>36.12</v>
       </c>
     </row>
     <row r="64">
@@ -1961,16 +2001,16 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>6.6</v>
+        <v>7.4</v>
       </c>
       <c r="F64" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G64" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H64" t="n">
-        <v>36.1</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="65">
@@ -1979,14 +2019,19 @@
           <t>2026-03-05</t>
         </is>
       </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E65" t="n">
-        <v>7.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F65" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G65" t="n">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="H65" t="n">
         <v>36.19</v>
@@ -1999,16 +2044,16 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>7.3</v>
+        <v>7</v>
       </c>
       <c r="F66" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G66" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="H66" t="n">
-        <v>36.13</v>
+        <v>36.14</v>
       </c>
     </row>
     <row r="67">
@@ -2018,16 +2063,16 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>7.6</v>
+        <v>6.9</v>
       </c>
       <c r="F67" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G67" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H67" t="n">
-        <v>36.12</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="68">
@@ -2043,17 +2088,27 @@
           <t>2026-03-09</t>
         </is>
       </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>high energy</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E69" t="n">
-        <v>8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F69" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G69" t="n">
         <v>64</v>
       </c>
       <c r="H69" t="n">
-        <v>36.13</v>
+        <v>36.14</v>
       </c>
     </row>
     <row r="70">
@@ -2071,13 +2126,13 @@
         <v>7.1</v>
       </c>
       <c r="F70" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G70" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H70" t="n">
-        <v>36.28</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="71">
@@ -2087,16 +2142,16 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="F71" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G71" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="H71" t="n">
-        <v>36.2</v>
+        <v>36.29</v>
       </c>
     </row>
     <row r="72">
@@ -2105,22 +2160,27 @@
           <t>2026-03-12</t>
         </is>
       </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>high energy</t>
+        </is>
+      </c>
       <c r="D72" t="inlineStr">
         <is>
           <t>great</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>7.1</v>
+        <v>7.8</v>
       </c>
       <c r="F72" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G72" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="H72" t="n">
-        <v>36.23</v>
+        <v>36.35</v>
       </c>
     </row>
     <row r="73">
@@ -2130,7 +2190,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>7.6</v>
+        <v>7.8</v>
       </c>
       <c r="F73" t="n">
         <v>61</v>
@@ -2148,17 +2208,22 @@
           <t>2026-03-14</t>
         </is>
       </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E74" t="n">
-        <v>8.199999999999999</v>
+        <v>7.9</v>
       </c>
       <c r="F74" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G74" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H74" t="n">
-        <v>36.45</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="75">
@@ -2168,16 +2233,16 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>7.9</v>
+        <v>7</v>
       </c>
       <c r="F75" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G75" t="n">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="H75" t="n">
-        <v>36.48</v>
+        <v>36.55</v>
       </c>
     </row>
     <row r="76">
@@ -2200,13 +2265,13 @@
         <v>5.9</v>
       </c>
       <c r="F76" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G76" t="n">
         <v>41</v>
       </c>
       <c r="H76" t="n">
-        <v>36.46</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="77">
@@ -2215,18 +2280,13 @@
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>poor sleep</t>
-        </is>
-      </c>
       <c r="D77" t="inlineStr">
         <is>
           <t>stressed</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="F77" t="n">
         <v>65</v>
@@ -2235,7 +2295,7 @@
         <v>42</v>
       </c>
       <c r="H77" t="n">
-        <v>36.5</v>
+        <v>36.47</v>
       </c>
     </row>
     <row r="78">
@@ -2246,20 +2306,20 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>stressed</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>6.1</v>
+        <v>5.7</v>
       </c>
       <c r="F78" t="n">
         <v>67</v>
       </c>
       <c r="G78" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H78" t="n">
-        <v>36.43</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="79">
@@ -2279,16 +2339,16 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="F79" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G79" t="n">
         <v>40</v>
       </c>
       <c r="H79" t="n">
-        <v>36.49</v>
+        <v>36.46</v>
       </c>
     </row>
     <row r="80">
@@ -2297,17 +2357,22 @@
           <t>2026-03-20</t>
         </is>
       </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>stressed</t>
+        </is>
+      </c>
       <c r="E80" t="n">
-        <v>5.4</v>
+        <v>6.4</v>
       </c>
       <c r="F80" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G80" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H80" t="n">
-        <v>36.49</v>
+        <v>36.54</v>
       </c>
     </row>
     <row r="81">
@@ -2316,17 +2381,27 @@
           <t>2026-03-21</t>
         </is>
       </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>poor sleep</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>stressed</t>
+        </is>
+      </c>
       <c r="E81" t="n">
-        <v>5.7</v>
+        <v>5.5</v>
       </c>
       <c r="F81" t="n">
         <v>65</v>
       </c>
       <c r="G81" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="H81" t="n">
-        <v>36.52</v>
+        <v>36.43</v>
       </c>
     </row>
     <row r="82">
@@ -2337,25 +2412,25 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>poor sleep</t>
+          <t>sore breasts</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>stressed</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="F82" t="n">
         <v>66</v>
       </c>
       <c r="G82" t="n">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="H82" t="n">
-        <v>36.53</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="83">
@@ -2366,25 +2441,25 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>cravings</t>
+          <t>sore breasts</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>irritable</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="F83" t="n">
         <v>62</v>
       </c>
       <c r="G83" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H83" t="n">
-        <v>36.54</v>
+        <v>36.48</v>
       </c>
     </row>
     <row r="84">
@@ -2395,7 +2470,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>bloating</t>
+          <t>poor sleep</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2404,7 +2479,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>5.4</v>
+        <v>6.2</v>
       </c>
       <c r="F84" t="n">
         <v>63</v>
@@ -2413,7 +2488,7 @@
         <v>49</v>
       </c>
       <c r="H84" t="n">
-        <v>36.28</v>
+        <v>36.26</v>
       </c>
     </row>
     <row r="85">
@@ -2422,14 +2497,24 @@
           <t>2026-03-25</t>
         </is>
       </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>headache</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E85" t="n">
-        <v>6.4</v>
+        <v>6.7</v>
       </c>
       <c r="F85" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G85" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H85" t="n">
         <v>36.28</v>
@@ -2446,22 +2531,27 @@
           <t>heavy</t>
         </is>
       </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>headache</t>
+        </is>
+      </c>
       <c r="D86" t="inlineStr">
         <is>
           <t>okay</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>7.5</v>
+        <v>7.1</v>
       </c>
       <c r="F86" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="G86" t="n">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="H86" t="n">
-        <v>36.21</v>
+        <v>36.23</v>
       </c>
     </row>
     <row r="87">
@@ -2475,27 +2565,22 @@
           <t>heavy</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>backache; low energy</t>
-        </is>
-      </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="F87" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G87" t="n">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="H87" t="n">
-        <v>36.15</v>
+        <v>36.21</v>
       </c>
     </row>
     <row r="88">
@@ -2515,16 +2600,16 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>7.2</v>
+        <v>6.7</v>
       </c>
       <c r="F88" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G88" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H88" t="n">
-        <v>36.11</v>
+        <v>36.05</v>
       </c>
     </row>
     <row r="89">
@@ -2540,20 +2625,20 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E89" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="F89" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="G89" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="H89" t="n">
-        <v>36.23</v>
+        <v>36.15</v>
       </c>
     </row>
     <row r="90">
@@ -2567,22 +2652,27 @@
           <t>spotting</t>
         </is>
       </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>low energy</t>
+        </is>
+      </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>6.8</v>
+        <v>7.9</v>
       </c>
       <c r="F90" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G90" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H90" t="n">
-        <v>36.21</v>
+        <v>36.16</v>
       </c>
     </row>
     <row r="91">
@@ -2592,16 +2682,16 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>6.7</v>
+        <v>7.1</v>
       </c>
       <c r="F91" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G91" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="H91" t="n">
-        <v>36.05</v>
+        <v>36.11</v>
       </c>
     </row>
     <row r="92">
@@ -2610,22 +2700,17 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>great</t>
-        </is>
-      </c>
       <c r="E92" t="n">
-        <v>7.2</v>
+        <v>6.7</v>
       </c>
       <c r="F92" t="n">
         <v>58</v>
       </c>
       <c r="G92" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H92" t="n">
-        <v>36.15</v>
+        <v>36.17</v>
       </c>
     </row>
     <row r="93">
@@ -2635,16 +2720,16 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>7.9</v>
+        <v>8.1</v>
       </c>
       <c r="F93" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G93" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="H93" t="n">
-        <v>36.16</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="94">
@@ -2654,16 +2739,16 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>7.1</v>
+        <v>7.9</v>
       </c>
       <c r="F94" t="n">
         <v>56</v>
       </c>
       <c r="G94" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="H94" t="n">
-        <v>36.11</v>
+        <v>36.14</v>
       </c>
     </row>
     <row r="95">
@@ -2673,16 +2758,16 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>6.7</v>
+        <v>6.9</v>
       </c>
       <c r="F95" t="n">
         <v>58</v>
       </c>
       <c r="G95" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="H95" t="n">
-        <v>36.17</v>
+        <v>36.09</v>
       </c>
     </row>
     <row r="96">
@@ -2692,16 +2777,16 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>8.1</v>
+        <v>7</v>
       </c>
       <c r="F96" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G96" t="n">
         <v>66</v>
       </c>
       <c r="H96" t="n">
-        <v>36.18</v>
+        <v>36.17</v>
       </c>
     </row>
     <row r="97">
@@ -2710,17 +2795,22 @@
           <t>2026-04-06</t>
         </is>
       </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>great</t>
+        </is>
+      </c>
       <c r="E97" t="n">
-        <v>7.9</v>
+        <v>7.5</v>
       </c>
       <c r="F97" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G97" t="n">
         <v>71</v>
       </c>
       <c r="H97" t="n">
-        <v>36.14</v>
+        <v>36.1</v>
       </c>
     </row>
     <row r="98">
@@ -2730,16 +2820,16 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>6.9</v>
+        <v>7.5</v>
       </c>
       <c r="F98" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G98" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="H98" t="n">
-        <v>36.1</v>
+        <v>36.17</v>
       </c>
     </row>
     <row r="99">
@@ -2748,17 +2838,27 @@
           <t>2026-04-08</t>
         </is>
       </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>increased libido</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E99" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F99" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G99" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H99" t="n">
-        <v>36.18</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="100">
@@ -2767,17 +2867,27 @@
           <t>2026-04-09</t>
         </is>
       </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>high energy; increased libido</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>great</t>
+        </is>
+      </c>
       <c r="E100" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="F100" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G100" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H100" t="n">
-        <v>36.17</v>
+        <v>36.25</v>
       </c>
     </row>
     <row r="101">
@@ -2786,14 +2896,24 @@
           <t>2026-04-10</t>
         </is>
       </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>high energy; increased libido</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E101" t="n">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="F101" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G101" t="n">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="H101" t="n">
         <v>36.3</v>
@@ -2805,17 +2925,27 @@
           <t>2026-04-11</t>
         </is>
       </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>high energy; increased libido</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E102" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="F102" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G102" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H102" t="n">
-        <v>36.33</v>
+        <v>36.28</v>
       </c>
     </row>
     <row r="103">
@@ -2828,13 +2958,13 @@
         <v>7.6</v>
       </c>
       <c r="F103" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G103" t="n">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H103" t="n">
-        <v>36.4</v>
+        <v>36.51</v>
       </c>
     </row>
     <row r="104">
@@ -2844,16 +2974,16 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="F104" t="n">
         <v>60</v>
       </c>
       <c r="G104" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H104" t="n">
-        <v>36.52</v>
+        <v>36.43</v>
       </c>
     </row>
     <row r="105">
@@ -2862,11 +2992,6 @@
           <t>2026-04-14</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>okay</t>
-        </is>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2886,10 +3011,10 @@
         <v>62</v>
       </c>
       <c r="G106" t="n">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="H106" t="n">
-        <v>36.4</v>
+        <v>36.46</v>
       </c>
     </row>
     <row r="107">
@@ -2898,22 +3023,17 @@
           <t>2026-04-16</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="E107" t="n">
-        <v>8.1</v>
+        <v>7.6</v>
       </c>
       <c r="F107" t="n">
+        <v>58</v>
+      </c>
+      <c r="G107" t="n">
         <v>60</v>
       </c>
-      <c r="G107" t="n">
-        <v>59</v>
-      </c>
       <c r="H107" t="n">
-        <v>36.55</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="108">
@@ -2923,16 +3043,16 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>8.300000000000001</v>
+        <v>7.1</v>
       </c>
       <c r="F108" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G108" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H108" t="n">
-        <v>36.46</v>
+        <v>36.55</v>
       </c>
     </row>
     <row r="109">
@@ -2947,16 +3067,16 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="F109" t="n">
+        <v>61</v>
+      </c>
+      <c r="G109" t="n">
         <v>62</v>
       </c>
-      <c r="G109" t="n">
-        <v>56</v>
-      </c>
       <c r="H109" t="n">
-        <v>36.51</v>
+        <v>36.45</v>
       </c>
     </row>
     <row r="110">
@@ -2966,16 +3086,16 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>7.4</v>
+        <v>7.7</v>
       </c>
       <c r="F110" t="n">
         <v>60</v>
       </c>
       <c r="G110" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="H110" t="n">
-        <v>36.42</v>
+        <v>36.45</v>
       </c>
     </row>
     <row r="111">
@@ -2986,25 +3106,25 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>headache</t>
+          <t>poor sleep</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>7.6</v>
+        <v>7.3</v>
       </c>
       <c r="F111" t="n">
         <v>61</v>
       </c>
       <c r="G111" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H111" t="n">
-        <v>36.44</v>
+        <v>36.46</v>
       </c>
     </row>
     <row r="112">
@@ -3020,20 +3140,20 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>7.9</v>
+        <v>7.6</v>
       </c>
       <c r="F112" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G112" t="n">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="H112" t="n">
-        <v>36.45</v>
+        <v>36.49</v>
       </c>
     </row>
     <row r="113">
@@ -3043,16 +3163,16 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>6.7</v>
+        <v>7.4</v>
       </c>
       <c r="F113" t="n">
         <v>61</v>
       </c>
       <c r="G113" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H113" t="n">
-        <v>36.47</v>
+        <v>36.46</v>
       </c>
     </row>
     <row r="114">
@@ -3063,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>cravings</t>
+          <t>bloating</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3072,16 +3192,16 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="F114" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G114" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H114" t="n">
-        <v>36.3</v>
+        <v>36.26</v>
       </c>
     </row>
     <row r="115">
@@ -3090,17 +3210,22 @@
           <t>2026-04-24</t>
         </is>
       </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
       <c r="E115" t="n">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="F115" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G115" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H115" t="n">
-        <v>36.37</v>
+        <v>36.35</v>
       </c>
     </row>
     <row r="116">
@@ -3116,7 +3241,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>backache</t>
+          <t>low energy</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3125,16 +3250,16 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>7.6</v>
+        <v>7.2</v>
       </c>
       <c r="F116" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G116" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H116" t="n">
-        <v>36.05</v>
+        <v>36.16</v>
       </c>
     </row>
     <row r="117">
@@ -3148,27 +3273,22 @@
           <t>heavy</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>backache; cramps</t>
-        </is>
-      </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E117" t="n">
-        <v>7.5</v>
+        <v>6.9</v>
       </c>
       <c r="F117" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G117" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="H117" t="n">
-        <v>36.1</v>
+        <v>36.09</v>
       </c>
     </row>
     <row r="118">
@@ -3184,25 +3304,25 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>cramps</t>
+          <t>backache</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>7.1</v>
+        <v>7.4</v>
       </c>
       <c r="F118" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G118" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H118" t="n">
-        <v>36.16</v>
+        <v>36.17</v>
       </c>
     </row>
     <row r="119">
@@ -3216,22 +3336,27 @@
           <t>light</t>
         </is>
       </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>low energy</t>
+        </is>
+      </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="F119" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G119" t="n">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="H119" t="n">
-        <v>36.11</v>
+        <v>36.14</v>
       </c>
     </row>
     <row r="120">
@@ -3245,22 +3370,27 @@
           <t>spotting</t>
         </is>
       </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>low energy</t>
+        </is>
+      </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E120" t="n">
-        <v>7.3</v>
+        <v>6.8</v>
       </c>
       <c r="F120" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G120" t="n">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H120" t="n">
-        <v>36.17</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="121">
@@ -3270,16 +3400,16 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
       <c r="F121" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G121" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H121" t="n">
-        <v>36.17</v>
+        <v>36.14</v>
       </c>
     </row>
     <row r="122">
@@ -3289,16 +3419,16 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>7.6</v>
+        <v>7.2</v>
       </c>
       <c r="F122" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G122" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="H122" t="n">
-        <v>36.17</v>
+        <v>36.03</v>
       </c>
     </row>
     <row r="123">
@@ -3307,22 +3437,17 @@
           <t>2026-05-02</t>
         </is>
       </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>great</t>
-        </is>
-      </c>
       <c r="E123" t="n">
-        <v>7.2</v>
+        <v>7.7</v>
       </c>
       <c r="F123" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G123" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="H123" t="n">
-        <v>36.13</v>
+        <v>36.17</v>
       </c>
     </row>
     <row r="124">
@@ -3331,17 +3456,22 @@
           <t>2026-05-03</t>
         </is>
       </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E124" t="n">
         <v>7.3</v>
       </c>
       <c r="F124" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G124" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="H124" t="n">
-        <v>36.09</v>
+        <v>36.14</v>
       </c>
     </row>
     <row r="125">
@@ -3351,16 +3481,16 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="F125" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G125" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="H125" t="n">
-        <v>36.27</v>
+        <v>36.09</v>
       </c>
     </row>
     <row r="126">
@@ -3373,13 +3503,13 @@
         <v>7.5</v>
       </c>
       <c r="F126" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G126" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H126" t="n">
-        <v>36.15</v>
+        <v>36.1</v>
       </c>
     </row>
     <row r="127">
@@ -3388,17 +3518,27 @@
           <t>2026-05-06</t>
         </is>
       </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>high energy; increased libido</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E127" t="n">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="F127" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G127" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="H127" t="n">
-        <v>36.13</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="128">
@@ -3409,7 +3549,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>high energy</t>
+          <t>high energy; increased libido</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -3418,16 +3558,16 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>6.9</v>
+        <v>8</v>
       </c>
       <c r="F128" t="n">
         <v>57</v>
       </c>
       <c r="G128" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H128" t="n">
-        <v>36.16</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="129">
@@ -3443,20 +3583,20 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>great</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E129" t="n">
-        <v>7.7</v>
+        <v>7.5</v>
       </c>
       <c r="F129" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G129" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H129" t="n">
-        <v>36.25</v>
+        <v>36.26</v>
       </c>
     </row>
     <row r="130">
@@ -3465,22 +3605,27 @@
           <t>2026-05-09</t>
         </is>
       </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>increased libido</t>
+        </is>
+      </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>great</t>
         </is>
       </c>
       <c r="E130" t="n">
-        <v>7</v>
+        <v>8.1</v>
       </c>
       <c r="F130" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G130" t="n">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="H130" t="n">
-        <v>36.34</v>
+        <v>36.33</v>
       </c>
     </row>
     <row r="131">
@@ -3490,16 +3635,16 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>7.7</v>
+        <v>7.9</v>
       </c>
       <c r="F131" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G131" t="n">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="H131" t="n">
-        <v>36.4</v>
+        <v>36.35</v>
       </c>
     </row>
     <row r="132">
@@ -3509,16 +3654,16 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>6.7</v>
+        <v>7.7</v>
       </c>
       <c r="F132" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G132" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="H132" t="n">
-        <v>36.42</v>
+        <v>36.46</v>
       </c>
     </row>
     <row r="133">
@@ -3528,16 +3673,16 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>8</v>
+        <v>7.2</v>
       </c>
       <c r="F133" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G133" t="n">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="H133" t="n">
-        <v>36.51</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="134">
@@ -3547,16 +3692,16 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>8.199999999999999</v>
+        <v>7.9</v>
       </c>
       <c r="F134" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G134" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H134" t="n">
-        <v>36.44</v>
+        <v>36.48</v>
       </c>
     </row>
     <row r="135">
@@ -3566,16 +3711,16 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>7.9</v>
+        <v>7.5</v>
       </c>
       <c r="F135" t="n">
         <v>61</v>
       </c>
       <c r="G135" t="n">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="H135" t="n">
-        <v>36.54</v>
+        <v>36.42</v>
       </c>
     </row>
     <row r="136">
@@ -3585,16 +3730,16 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="F136" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G136" t="n">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="H136" t="n">
-        <v>36.36</v>
+        <v>36.47</v>
       </c>
     </row>
     <row r="137">
@@ -3603,22 +3748,17 @@
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="D137" t="inlineStr">
-        <is>
-          <t>okay</t>
-        </is>
-      </c>
       <c r="E137" t="n">
-        <v>7.4</v>
+        <v>7.8</v>
       </c>
       <c r="F137" t="n">
         <v>61</v>
       </c>
       <c r="G137" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="H137" t="n">
-        <v>36.53</v>
+        <v>36.57</v>
       </c>
     </row>
     <row r="138">
@@ -3627,17 +3767,22 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E138" t="n">
-        <v>7.2</v>
+        <v>6.8</v>
       </c>
       <c r="F138" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G138" t="n">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="H138" t="n">
-        <v>36.57</v>
+        <v>36.47</v>
       </c>
     </row>
     <row r="139">
@@ -3646,27 +3791,17 @@
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>bloating</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="E139" t="n">
-        <v>7.8</v>
+        <v>7.6</v>
       </c>
       <c r="F139" t="n">
         <v>62</v>
       </c>
       <c r="G139" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H139" t="n">
-        <v>36.48</v>
+        <v>36.46</v>
       </c>
     </row>
     <row r="140">
@@ -3675,27 +3810,22 @@
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>cravings</t>
-        </is>
-      </c>
       <c r="D140" t="inlineStr">
         <is>
           <t>okay</t>
         </is>
       </c>
       <c r="E140" t="n">
-        <v>7.6</v>
+        <v>7</v>
       </c>
       <c r="F140" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G140" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="H140" t="n">
-        <v>36.46</v>
+        <v>36.48</v>
       </c>
     </row>
     <row r="141">
@@ -3704,27 +3834,22 @@
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>bloating</t>
-        </is>
-      </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E141" t="n">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="F141" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G141" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H141" t="n">
-        <v>36.55</v>
+        <v>36.54</v>
       </c>
     </row>
     <row r="142">
@@ -3735,7 +3860,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>poor sleep</t>
+          <t>headache</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -3747,13 +3872,13 @@
         <v>6.8</v>
       </c>
       <c r="F142" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G142" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="H142" t="n">
-        <v>36.27</v>
+        <v>36.36</v>
       </c>
     </row>
     <row r="143">
@@ -3764,17 +3889,17 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>irritable</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E143" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="F143" t="n">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G143" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H143" t="n">
         <v>36.28</v>
@@ -3797,16 +3922,16 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>7.8</v>
+        <v>6.9</v>
       </c>
       <c r="F144" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G144" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H144" t="n">
-        <v>36.16</v>
+        <v>36.25</v>
       </c>
     </row>
     <row r="145">
@@ -3822,25 +3947,25 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>backache; headache</t>
+          <t>cramps</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E145" t="n">
-        <v>7.1</v>
+        <v>8</v>
       </c>
       <c r="F145" t="n">
         <v>56</v>
       </c>
       <c r="G145" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H145" t="n">
-        <v>36.02</v>
+        <v>36.06</v>
       </c>
     </row>
     <row r="146">
@@ -3856,20 +3981,20 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>7.2</v>
+        <v>6.7</v>
       </c>
       <c r="F146" t="n">
         <v>57</v>
       </c>
       <c r="G146" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H146" t="n">
-        <v>36.14</v>
+        <v>36.21</v>
       </c>
     </row>
     <row r="147">
@@ -3883,27 +4008,22 @@
           <t>light</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>low energy</t>
-        </is>
-      </c>
       <c r="D147" t="inlineStr">
         <is>
           <t>okay</t>
         </is>
       </c>
       <c r="E147" t="n">
-        <v>7.7</v>
+        <v>7.4</v>
       </c>
       <c r="F147" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G147" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H147" t="n">
-        <v>36.1</v>
+        <v>36.23</v>
       </c>
     </row>
     <row r="148">
@@ -3917,27 +4037,22 @@
           <t>spotting</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>low energy</t>
-        </is>
-      </c>
       <c r="D148" t="inlineStr">
         <is>
           <t>okay</t>
         </is>
       </c>
       <c r="E148" t="n">
-        <v>7.7</v>
+        <v>7.3</v>
       </c>
       <c r="F148" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G148" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H148" t="n">
-        <v>36.22</v>
+        <v>36.19</v>
       </c>
     </row>
     <row r="149">
@@ -3947,16 +4062,16 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>6.6</v>
+        <v>7.6</v>
       </c>
       <c r="F149" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G149" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H149" t="n">
-        <v>36.11</v>
+        <v>36.15</v>
       </c>
     </row>
     <row r="150">
@@ -3966,16 +4081,16 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>7.1</v>
+        <v>7.4</v>
       </c>
       <c r="F150" t="n">
         <v>57</v>
       </c>
       <c r="G150" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H150" t="n">
-        <v>36.21</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="151">
@@ -3984,11 +4099,6 @@
           <t>2026-05-30</t>
         </is>
       </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -3997,16 +4107,16 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>6.8</v>
+        <v>7.4</v>
       </c>
       <c r="F152" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G152" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="H152" t="n">
-        <v>36.1</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="153">
@@ -4015,22 +4125,17 @@
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="E153" t="n">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
       <c r="F153" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G153" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H153" t="n">
-        <v>36.18</v>
+        <v>36.12</v>
       </c>
     </row>
     <row r="154">
@@ -4041,20 +4146,20 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E154" t="n">
         <v>7.6</v>
       </c>
       <c r="F154" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G154" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="H154" t="n">
-        <v>36.17</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="155">
@@ -4063,17 +4168,22 @@
           <t>2026-06-03</t>
         </is>
       </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E155" t="n">
-        <v>7.1</v>
+        <v>6.9</v>
       </c>
       <c r="F155" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="G155" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="H155" t="n">
-        <v>36.05</v>
+        <v>36.04</v>
       </c>
     </row>
     <row r="156">
@@ -4082,17 +4192,22 @@
           <t>2026-06-04</t>
         </is>
       </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E156" t="n">
-        <v>7.6</v>
+        <v>7.3</v>
       </c>
       <c r="F156" t="n">
         <v>57</v>
       </c>
       <c r="G156" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H156" t="n">
-        <v>36.18</v>
+        <v>36.22</v>
       </c>
     </row>
     <row r="157">
@@ -4101,22 +4216,27 @@
           <t>2026-06-05</t>
         </is>
       </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>high energy</t>
+        </is>
+      </c>
       <c r="D157" t="inlineStr">
         <is>
           <t>great</t>
         </is>
       </c>
       <c r="E157" t="n">
-        <v>7.2</v>
+        <v>7.9</v>
       </c>
       <c r="F157" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G157" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="H157" t="n">
-        <v>36.23</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="158">
@@ -4125,17 +4245,27 @@
           <t>2026-06-06</t>
         </is>
       </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>high energy</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>great</t>
+        </is>
+      </c>
       <c r="E158" t="n">
-        <v>7.3</v>
+        <v>7.4</v>
       </c>
       <c r="F158" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G158" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H158" t="n">
-        <v>36.28</v>
+        <v>36.34</v>
       </c>
     </row>
     <row r="159">
@@ -4144,17 +4274,27 @@
           <t>2026-06-07</t>
         </is>
       </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>increased libido</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E159" t="n">
-        <v>7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F159" t="n">
         <v>57</v>
       </c>
       <c r="G159" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H159" t="n">
-        <v>36.35</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="160">
@@ -4164,16 +4304,16 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>6</v>
+        <v>7.8</v>
       </c>
       <c r="F160" t="n">
         <v>62</v>
       </c>
       <c r="G160" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="H160" t="n">
-        <v>36.46</v>
+        <v>36.48</v>
       </c>
     </row>
     <row r="161">
@@ -4186,13 +4326,13 @@
         <v>7.3</v>
       </c>
       <c r="F161" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G161" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="H161" t="n">
-        <v>36.53</v>
+        <v>36.47</v>
       </c>
     </row>
     <row r="162">
@@ -4201,11 +4341,6 @@
           <t>2026-06-10</t>
         </is>
       </c>
-      <c r="D162" t="inlineStr">
-        <is>
-          <t>okay</t>
-        </is>
-      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -4214,16 +4349,16 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F163" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G163" t="n">
         <v>60</v>
       </c>
       <c r="H163" t="n">
-        <v>36.48</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="164">
@@ -4232,17 +4367,22 @@
           <t>2026-06-12</t>
         </is>
       </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E164" t="n">
-        <v>6.8</v>
+        <v>7.4</v>
       </c>
       <c r="F164" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G164" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="H164" t="n">
-        <v>36.47</v>
+        <v>36.55</v>
       </c>
     </row>
     <row r="165">
@@ -4252,16 +4392,16 @@
         </is>
       </c>
       <c r="E165" t="n">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
       <c r="F165" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G165" t="n">
         <v>59</v>
       </c>
       <c r="H165" t="n">
-        <v>36.47</v>
+        <v>36.48</v>
       </c>
     </row>
     <row r="166">
@@ -4271,16 +4411,16 @@
         </is>
       </c>
       <c r="E166" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="F166" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="G166" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H166" t="n">
-        <v>36.48</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="167">
@@ -4290,13 +4430,13 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>7.3</v>
+        <v>7.4</v>
       </c>
       <c r="F167" t="n">
         <v>61</v>
       </c>
       <c r="G167" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="H167" t="n">
         <v>36.46</v>
@@ -4310,25 +4450,25 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>headache</t>
+          <t>sore breasts</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E168" t="n">
-        <v>7.7</v>
+        <v>7.5</v>
       </c>
       <c r="F168" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G168" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H168" t="n">
-        <v>36.56</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="169">
@@ -4337,17 +4477,27 @@
           <t>2026-06-17</t>
         </is>
       </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>sore breasts</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E169" t="n">
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="F169" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G169" t="n">
         <v>57</v>
       </c>
       <c r="H169" t="n">
-        <v>36.46</v>
+        <v>36.48</v>
       </c>
     </row>
     <row r="170">
@@ -4363,20 +4513,20 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>irritable</t>
         </is>
       </c>
       <c r="E170" t="n">
-        <v>6.7</v>
+        <v>7.2</v>
       </c>
       <c r="F170" t="n">
         <v>61</v>
       </c>
       <c r="G170" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="H170" t="n">
-        <v>36.58</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="171">
@@ -4385,27 +4535,17 @@
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>bloating</t>
-        </is>
-      </c>
-      <c r="D171" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
       <c r="E171" t="n">
-        <v>7.1</v>
+        <v>6.5</v>
       </c>
       <c r="F171" t="n">
         <v>64</v>
       </c>
       <c r="G171" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="H171" t="n">
-        <v>36.27</v>
+        <v>36.36</v>
       </c>
     </row>
     <row r="172">
@@ -4416,25 +4556,25 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>poor sleep</t>
+          <t>bloating</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>irritable</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E172" t="n">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="F172" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G172" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="H172" t="n">
-        <v>36.39</v>
+        <v>36.32</v>
       </c>
     </row>
     <row r="173">
@@ -4448,27 +4588,22 @@
           <t>heavy</t>
         </is>
       </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>headache</t>
-        </is>
-      </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E173" t="n">
-        <v>7.7</v>
+        <v>7.5</v>
       </c>
       <c r="F173" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G173" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="H173" t="n">
-        <v>36.26</v>
+        <v>36.21</v>
       </c>
     </row>
     <row r="174">
@@ -4482,27 +4617,22 @@
           <t>heavy</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>low energy; backache</t>
-        </is>
-      </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E174" t="n">
         <v>7.6</v>
       </c>
       <c r="F174" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G174" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H174" t="n">
-        <v>36.2</v>
+        <v>36.15</v>
       </c>
     </row>
     <row r="175">
@@ -4516,27 +4646,22 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>cramps</t>
-        </is>
-      </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E175" t="n">
-        <v>8.300000000000001</v>
+        <v>7.7</v>
       </c>
       <c r="F175" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G175" t="n">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="H175" t="n">
-        <v>36.19</v>
+        <v>36.16</v>
       </c>
     </row>
     <row r="176">
@@ -4556,16 +4681,16 @@
         </is>
       </c>
       <c r="E176" t="n">
-        <v>7</v>
+        <v>7.8</v>
       </c>
       <c r="F176" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G176" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="H176" t="n">
-        <v>36.21</v>
+        <v>36.09</v>
       </c>
     </row>
     <row r="177">
@@ -4579,27 +4704,22 @@
           <t>spotting</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>low energy</t>
-        </is>
-      </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E177" t="n">
-        <v>7.1</v>
+        <v>7.4</v>
       </c>
       <c r="F177" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G177" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="H177" t="n">
-        <v>36.14</v>
+        <v>36.13</v>
       </c>
     </row>
     <row r="178">
@@ -4608,17 +4728,22 @@
           <t>2026-06-26</t>
         </is>
       </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E178" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="F178" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G178" t="n">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="H178" t="n">
-        <v>36.18</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="179">
@@ -4627,17 +4752,22 @@
           <t>2026-06-27</t>
         </is>
       </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E179" t="n">
-        <v>7.5</v>
+        <v>7.2</v>
       </c>
       <c r="F179" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G179" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="H179" t="n">
-        <v>36.18</v>
+        <v>36.16</v>
       </c>
     </row>
     <row r="180">
@@ -4647,16 +4777,16 @@
         </is>
       </c>
       <c r="E180" t="n">
-        <v>6.9</v>
+        <v>7.4</v>
       </c>
       <c r="F180" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G180" t="n">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="H180" t="n">
-        <v>36.17</v>
+        <v>36.25</v>
       </c>
     </row>
     <row r="181">
@@ -4666,16 +4796,16 @@
         </is>
       </c>
       <c r="E181" t="n">
-        <v>8.1</v>
+        <v>7.9</v>
       </c>
       <c r="F181" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G181" t="n">
         <v>67</v>
       </c>
       <c r="H181" t="n">
-        <v>36.17</v>
+        <v>36.16</v>
       </c>
     </row>
     <row r="182">
@@ -4690,16 +4820,16 @@
         </is>
       </c>
       <c r="E182" t="n">
-        <v>7.3</v>
+        <v>6.6</v>
       </c>
       <c r="F182" t="n">
         <v>59</v>
       </c>
       <c r="G182" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H182" t="n">
-        <v>36.12</v>
+        <v>36.16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync workshop test data from source of truth (#2)
Refresh the served datasets to match female-health/landing (the source
of truth). The live workshop was serving a pre-strengthening dataset.

- cycle_test_data.csv: ovulation signals now in most cycles
  (high energy 3 -> 13 days, added "increased libido"); 91 -> 109 rows
- wearable_test_data.csv: deeper luteal HRV dip (follicular-high ->
  luteal-low -> pre-period crash)
- merged_test_data.csv + .xlsx: regenerated answer key to match
- index.html: update FILE 1 download-card label (91 rows, 2 KB ->
  109 rows, 3 KB); wearable card unchanged (still 176 rows, 5 KB)

Page structure, prompts and expected-result descriptions unchanged.


Claude-Session: https://claude.ai/code/session_012wFqHjHyYrz8x44QT9Sbrq

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/merged_test_data.xlsx
+++ b/merged_test_data.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="merged" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="merged" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -759,16 +759,16 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>8.1</v>
+        <v>7.4</v>
       </c>
       <c r="F13" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G13" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H13" t="n">
-        <v>36.1</v>
+        <v>36.13</v>
       </c>
     </row>
     <row r="14">
@@ -777,17 +777,22 @@
           <t>2026-01-13</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>great</t>
+        </is>
+      </c>
       <c r="E14" t="n">
-        <v>7.5</v>
+        <v>7.1</v>
       </c>
       <c r="F14" t="n">
         <v>57</v>
       </c>
       <c r="G14" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="H14" t="n">
-        <v>36.15</v>
+        <v>36.26</v>
       </c>
     </row>
     <row r="15">
@@ -796,17 +801,22 @@
           <t>2026-01-14</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E15" t="n">
-        <v>7.3</v>
+        <v>6.8</v>
       </c>
       <c r="F15" t="n">
         <v>57</v>
       </c>
       <c r="G15" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H15" t="n">
-        <v>36.19</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="16">
@@ -816,16 +826,16 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="F16" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G16" t="n">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="H16" t="n">
-        <v>36.35</v>
+        <v>36.34</v>
       </c>
     </row>
     <row r="17">
@@ -835,16 +845,16 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>6.9</v>
+        <v>7</v>
       </c>
       <c r="F17" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G17" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="H17" t="n">
-        <v>36.47</v>
+        <v>36.53</v>
       </c>
     </row>
     <row r="18">
@@ -853,17 +863,22 @@
           <t>2026-01-17</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E18" t="n">
-        <v>7.4</v>
+        <v>7</v>
       </c>
       <c r="F18" t="n">
         <v>61</v>
       </c>
       <c r="G18" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H18" t="n">
-        <v>36.55</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="19">
@@ -872,14 +887,19 @@
           <t>2026-01-18</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E19" t="n">
-        <v>7.6</v>
+        <v>7.3</v>
       </c>
       <c r="F19" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G19" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H19" t="n">
         <v>36.55</v>
@@ -893,20 +913,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>7.8</v>
+        <v>7.2</v>
       </c>
       <c r="F20" t="n">
         <v>60</v>
       </c>
       <c r="G20" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H20" t="n">
-        <v>36.39</v>
+        <v>36.43</v>
       </c>
     </row>
     <row r="21">
@@ -915,17 +935,22 @@
           <t>2026-01-20</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E21" t="n">
-        <v>6.9</v>
+        <v>6.4</v>
       </c>
       <c r="F21" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G21" t="n">
         <v>58</v>
       </c>
       <c r="H21" t="n">
-        <v>36.5</v>
+        <v>36.47</v>
       </c>
     </row>
     <row r="22">
@@ -935,16 +960,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>7.3</v>
+        <v>6.9</v>
       </c>
       <c r="F22" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G22" t="n">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="H22" t="n">
-        <v>36.42</v>
+        <v>36.52</v>
       </c>
     </row>
     <row r="23">
@@ -953,22 +978,17 @@
           <t>2026-01-22</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="E23" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="F23" t="n">
+        <v>62</v>
+      </c>
+      <c r="G23" t="n">
         <v>63</v>
       </c>
-      <c r="G23" t="n">
-        <v>67</v>
-      </c>
       <c r="H23" t="n">
-        <v>36.51</v>
+        <v>36.56</v>
       </c>
     </row>
     <row r="24">
@@ -977,22 +997,17 @@
           <t>2026-01-23</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="E24" t="n">
-        <v>6.5</v>
+        <v>7.4</v>
       </c>
       <c r="F24" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G24" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H24" t="n">
-        <v>36.44</v>
+        <v>36.42</v>
       </c>
     </row>
     <row r="25">
@@ -1003,7 +1018,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>poor sleep</t>
+          <t>bloating</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1012,16 +1027,16 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>8.1</v>
+        <v>6.7</v>
       </c>
       <c r="F25" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G25" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H25" t="n">
-        <v>36.55</v>
+        <v>36.58</v>
       </c>
     </row>
     <row r="26">
@@ -1030,27 +1045,17 @@
           <t>2026-01-25</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>bloating</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>okay</t>
-        </is>
-      </c>
       <c r="E26" t="n">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="F26" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G26" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H26" t="n">
-        <v>36.47</v>
+        <v>36.48</v>
       </c>
     </row>
     <row r="27">
@@ -1061,25 +1066,25 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>sore breasts</t>
+          <t>headache</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="F27" t="n">
         <v>62</v>
       </c>
       <c r="G27" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="H27" t="n">
-        <v>36.39</v>
+        <v>36.53</v>
       </c>
     </row>
     <row r="28">
@@ -1088,17 +1093,22 @@
           <t>2026-01-27</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
       <c r="E28" t="n">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="F28" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G28" t="n">
         <v>48</v>
       </c>
       <c r="H28" t="n">
-        <v>36.33</v>
+        <v>36.28</v>
       </c>
     </row>
     <row r="29">
@@ -1107,13 +1117,18 @@
           <t>2026-01-28</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>bloating</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="F29" t="n">
         <v>62</v>
@@ -1122,7 +1137,7 @@
         <v>45</v>
       </c>
       <c r="H29" t="n">
-        <v>36.29</v>
+        <v>36.31</v>
       </c>
     </row>
     <row r="30">
@@ -1147,16 +1162,16 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>8.199999999999999</v>
+        <v>7.1</v>
       </c>
       <c r="F30" t="n">
         <v>57</v>
       </c>
       <c r="G30" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H30" t="n">
-        <v>36.22</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="31">
@@ -1170,22 +1185,27 @@
           <t>heavy</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>backache</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>7.9</v>
+        <v>7.7</v>
       </c>
       <c r="F31" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G31" t="n">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="H31" t="n">
-        <v>36.13</v>
+        <v>36.16</v>
       </c>
     </row>
     <row r="32">
@@ -1205,16 +1225,16 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>7.7</v>
+        <v>7.6</v>
       </c>
       <c r="F32" t="n">
         <v>58</v>
       </c>
       <c r="G32" t="n">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="H32" t="n">
-        <v>36.16</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="33">
@@ -1234,13 +1254,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>7.6</v>
+        <v>7.4</v>
       </c>
       <c r="F33" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G33" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="H33" t="n">
         <v>36.18</v>
@@ -1263,16 +1283,16 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="F34" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G34" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H34" t="n">
-        <v>36.18</v>
+        <v>36.06</v>
       </c>
     </row>
     <row r="35">
@@ -1282,16 +1302,16 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="F35" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G35" t="n">
         <v>69</v>
       </c>
       <c r="H35" t="n">
-        <v>36.06</v>
+        <v>36.1</v>
       </c>
     </row>
     <row r="36">
@@ -1300,17 +1320,22 @@
           <t>2026-02-04</t>
         </is>
       </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E36" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="F36" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G36" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="H36" t="n">
-        <v>36.1</v>
+        <v>36.15</v>
       </c>
     </row>
     <row r="37">
@@ -1325,13 +1350,13 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="F37" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G37" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H37" t="n">
         <v>36.15</v>
@@ -1343,22 +1368,17 @@
           <t>2026-02-06</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>okay</t>
-        </is>
-      </c>
       <c r="E38" t="n">
-        <v>7.5</v>
+        <v>7.6</v>
       </c>
       <c r="F38" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G38" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H38" t="n">
-        <v>36.15</v>
+        <v>36.17</v>
       </c>
     </row>
     <row r="39">
@@ -1367,17 +1387,22 @@
           <t>2026-02-07</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E39" t="n">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="F39" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G39" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H39" t="n">
-        <v>36.17</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="40">
@@ -1386,22 +1411,17 @@
           <t>2026-02-08</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>okay</t>
-        </is>
-      </c>
       <c r="E40" t="n">
         <v>7.5</v>
       </c>
       <c r="F40" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G40" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H40" t="n">
-        <v>36.18</v>
+        <v>36.15</v>
       </c>
     </row>
     <row r="41">
@@ -1410,17 +1430,22 @@
           <t>2026-02-09</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E41" t="n">
-        <v>7.5</v>
+        <v>7.1</v>
       </c>
       <c r="F41" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G41" t="n">
         <v>70</v>
       </c>
       <c r="H41" t="n">
-        <v>36.15</v>
+        <v>36.02</v>
       </c>
     </row>
     <row r="42">
@@ -1429,9 +1454,14 @@
           <t>2026-02-10</t>
         </is>
       </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>high energy</t>
+        </is>
+      </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
     </row>
@@ -1441,17 +1471,27 @@
           <t>2026-02-11</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>high energy</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>great</t>
+        </is>
+      </c>
       <c r="E43" t="n">
-        <v>7.1</v>
+        <v>7.4</v>
       </c>
       <c r="F43" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G43" t="n">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H43" t="n">
-        <v>36.24</v>
+        <v>36.15</v>
       </c>
     </row>
     <row r="44">
@@ -1460,22 +1500,27 @@
           <t>2026-02-12</t>
         </is>
       </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>high energy</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>great</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>7.4</v>
+        <v>7.8</v>
       </c>
       <c r="F44" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G44" t="n">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="H44" t="n">
-        <v>36.2</v>
+        <v>36.22</v>
       </c>
     </row>
     <row r="45">
@@ -1484,27 +1529,22 @@
           <t>2026-02-13</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>high energy</t>
-        </is>
-      </c>
       <c r="D45" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="F45" t="n">
         <v>58</v>
       </c>
       <c r="G45" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="H45" t="n">
-        <v>36.4</v>
+        <v>36.27</v>
       </c>
     </row>
     <row r="46">
@@ -1513,17 +1553,22 @@
           <t>2026-02-14</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E46" t="n">
-        <v>7.8</v>
+        <v>7.5</v>
       </c>
       <c r="F46" t="n">
+        <v>61</v>
+      </c>
+      <c r="G46" t="n">
         <v>58</v>
       </c>
-      <c r="G46" t="n">
-        <v>59</v>
-      </c>
       <c r="H46" t="n">
-        <v>36.42</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="47">
@@ -1532,22 +1577,17 @@
           <t>2026-02-15</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="E47" t="n">
-        <v>7.9</v>
+        <v>7.5</v>
       </c>
       <c r="F47" t="n">
         <v>61</v>
       </c>
       <c r="G47" t="n">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="H47" t="n">
-        <v>36.49</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="48">
@@ -1556,22 +1596,17 @@
           <t>2026-02-16</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>okay</t>
-        </is>
-      </c>
       <c r="E48" t="n">
-        <v>6.8</v>
+        <v>7.1</v>
       </c>
       <c r="F48" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G48" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="H48" t="n">
-        <v>36.54</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="49">
@@ -1581,16 +1616,16 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>7.9</v>
+        <v>6.9</v>
       </c>
       <c r="F49" t="n">
+        <v>61</v>
+      </c>
+      <c r="G49" t="n">
         <v>62</v>
       </c>
-      <c r="G49" t="n">
-        <v>56</v>
-      </c>
       <c r="H49" t="n">
-        <v>36.53</v>
+        <v>36.43</v>
       </c>
     </row>
     <row r="50">
@@ -1599,8 +1634,13 @@
           <t>2026-02-18</t>
         </is>
       </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E50" t="n">
-        <v>6.9</v>
+        <v>7.3</v>
       </c>
       <c r="F50" t="n">
         <v>61</v>
@@ -1609,7 +1649,7 @@
         <v>59</v>
       </c>
       <c r="H50" t="n">
-        <v>36.5</v>
+        <v>36.45</v>
       </c>
     </row>
     <row r="51">
@@ -1618,14 +1658,19 @@
           <t>2026-02-19</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E51" t="n">
-        <v>7.5</v>
+        <v>6.8</v>
       </c>
       <c r="F51" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G51" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="H51" t="n">
         <v>36.51</v>
@@ -1638,16 +1683,16 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
       <c r="F52" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G52" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H52" t="n">
-        <v>36.54</v>
+        <v>36.42</v>
       </c>
     </row>
     <row r="53">
@@ -1656,17 +1701,22 @@
           <t>2026-02-21</t>
         </is>
       </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E53" t="n">
-        <v>7.8</v>
+        <v>7.4</v>
       </c>
       <c r="F53" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G53" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="H53" t="n">
-        <v>36.54</v>
+        <v>36.53</v>
       </c>
     </row>
     <row r="54">
@@ -1676,16 +1726,16 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>7.5</v>
+        <v>7.3</v>
       </c>
       <c r="F54" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G54" t="n">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="H54" t="n">
-        <v>36.47</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="55">
@@ -1694,27 +1744,17 @@
           <t>2026-02-23</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>cravings</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
       <c r="E55" t="n">
-        <v>7.3</v>
+        <v>7</v>
       </c>
       <c r="F55" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G55" t="n">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="H55" t="n">
-        <v>36.54</v>
+        <v>36.41</v>
       </c>
     </row>
     <row r="56">
@@ -1725,25 +1765,25 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>sore breasts</t>
+          <t>cravings</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>irritable</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>6.2</v>
+        <v>6.4</v>
       </c>
       <c r="F56" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G56" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="H56" t="n">
-        <v>36.51</v>
+        <v>36.56</v>
       </c>
     </row>
     <row r="57">
@@ -1752,27 +1792,17 @@
           <t>2026-02-25</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>headache</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>irritable</t>
-        </is>
-      </c>
       <c r="E57" t="n">
-        <v>6.6</v>
+        <v>7.1</v>
       </c>
       <c r="F57" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G57" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="H57" t="n">
-        <v>36.34</v>
+        <v>36.29</v>
       </c>
     </row>
     <row r="58">
@@ -1783,25 +1813,25 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>headache</t>
+          <t>bloating</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>6.8</v>
+        <v>6.2</v>
       </c>
       <c r="F58" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G58" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="H58" t="n">
-        <v>36.33</v>
+        <v>36.34</v>
       </c>
     </row>
     <row r="59">
@@ -1815,22 +1845,27 @@
           <t>heavy</t>
         </is>
       </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>backache</t>
+        </is>
+      </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>7.4</v>
+        <v>7.8</v>
       </c>
       <c r="F59" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G59" t="n">
         <v>65</v>
       </c>
       <c r="H59" t="n">
-        <v>36.14</v>
+        <v>36.08</v>
       </c>
     </row>
     <row r="60">
@@ -1844,22 +1879,27 @@
           <t>heavy</t>
         </is>
       </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>backache</t>
+        </is>
+      </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>8.1</v>
+        <v>7.2</v>
       </c>
       <c r="F60" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G60" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H60" t="n">
-        <v>36.04</v>
+        <v>36.21</v>
       </c>
     </row>
     <row r="61">
@@ -1875,25 +1915,25 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>low energy</t>
+          <t>headache</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>7.7</v>
+        <v>7.3</v>
       </c>
       <c r="F61" t="n">
         <v>57</v>
       </c>
       <c r="G61" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="H61" t="n">
-        <v>36.17</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="62">
@@ -1909,20 +1949,20 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>7.2</v>
+        <v>6.8</v>
       </c>
       <c r="F62" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G62" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="H62" t="n">
-        <v>36.13</v>
+        <v>36.07</v>
       </c>
     </row>
     <row r="63">
@@ -1942,16 +1982,16 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>6.8</v>
+        <v>7.3</v>
       </c>
       <c r="F63" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G63" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H63" t="n">
-        <v>36.05</v>
+        <v>36.12</v>
       </c>
     </row>
     <row r="64">
@@ -1961,16 +2001,16 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>6.6</v>
+        <v>7.4</v>
       </c>
       <c r="F64" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G64" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H64" t="n">
-        <v>36.1</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="65">
@@ -1979,14 +2019,19 @@
           <t>2026-03-05</t>
         </is>
       </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E65" t="n">
-        <v>7.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F65" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G65" t="n">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="H65" t="n">
         <v>36.19</v>
@@ -1999,16 +2044,16 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>7.3</v>
+        <v>7</v>
       </c>
       <c r="F66" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G66" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="H66" t="n">
-        <v>36.13</v>
+        <v>36.14</v>
       </c>
     </row>
     <row r="67">
@@ -2018,16 +2063,16 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>7.6</v>
+        <v>6.9</v>
       </c>
       <c r="F67" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G67" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H67" t="n">
-        <v>36.12</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="68">
@@ -2043,17 +2088,27 @@
           <t>2026-03-09</t>
         </is>
       </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>high energy</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E69" t="n">
-        <v>8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F69" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G69" t="n">
         <v>64</v>
       </c>
       <c r="H69" t="n">
-        <v>36.13</v>
+        <v>36.14</v>
       </c>
     </row>
     <row r="70">
@@ -2071,13 +2126,13 @@
         <v>7.1</v>
       </c>
       <c r="F70" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G70" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H70" t="n">
-        <v>36.28</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="71">
@@ -2087,16 +2142,16 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="F71" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G71" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="H71" t="n">
-        <v>36.2</v>
+        <v>36.29</v>
       </c>
     </row>
     <row r="72">
@@ -2105,22 +2160,27 @@
           <t>2026-03-12</t>
         </is>
       </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>high energy</t>
+        </is>
+      </c>
       <c r="D72" t="inlineStr">
         <is>
           <t>great</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>7.1</v>
+        <v>7.8</v>
       </c>
       <c r="F72" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G72" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="H72" t="n">
-        <v>36.23</v>
+        <v>36.35</v>
       </c>
     </row>
     <row r="73">
@@ -2130,7 +2190,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>7.6</v>
+        <v>7.8</v>
       </c>
       <c r="F73" t="n">
         <v>61</v>
@@ -2148,17 +2208,22 @@
           <t>2026-03-14</t>
         </is>
       </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E74" t="n">
-        <v>8.199999999999999</v>
+        <v>7.9</v>
       </c>
       <c r="F74" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G74" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H74" t="n">
-        <v>36.45</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="75">
@@ -2168,16 +2233,16 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>7.9</v>
+        <v>7</v>
       </c>
       <c r="F75" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G75" t="n">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="H75" t="n">
-        <v>36.48</v>
+        <v>36.55</v>
       </c>
     </row>
     <row r="76">
@@ -2200,13 +2265,13 @@
         <v>5.9</v>
       </c>
       <c r="F76" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G76" t="n">
         <v>41</v>
       </c>
       <c r="H76" t="n">
-        <v>36.46</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="77">
@@ -2215,18 +2280,13 @@
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>poor sleep</t>
-        </is>
-      </c>
       <c r="D77" t="inlineStr">
         <is>
           <t>stressed</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="F77" t="n">
         <v>65</v>
@@ -2235,7 +2295,7 @@
         <v>42</v>
       </c>
       <c r="H77" t="n">
-        <v>36.5</v>
+        <v>36.47</v>
       </c>
     </row>
     <row r="78">
@@ -2246,20 +2306,20 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>stressed</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>6.1</v>
+        <v>5.7</v>
       </c>
       <c r="F78" t="n">
         <v>67</v>
       </c>
       <c r="G78" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H78" t="n">
-        <v>36.43</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="79">
@@ -2279,16 +2339,16 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="F79" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G79" t="n">
         <v>40</v>
       </c>
       <c r="H79" t="n">
-        <v>36.49</v>
+        <v>36.46</v>
       </c>
     </row>
     <row r="80">
@@ -2297,17 +2357,22 @@
           <t>2026-03-20</t>
         </is>
       </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>stressed</t>
+        </is>
+      </c>
       <c r="E80" t="n">
-        <v>5.4</v>
+        <v>6.4</v>
       </c>
       <c r="F80" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G80" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H80" t="n">
-        <v>36.49</v>
+        <v>36.54</v>
       </c>
     </row>
     <row r="81">
@@ -2316,17 +2381,27 @@
           <t>2026-03-21</t>
         </is>
       </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>poor sleep</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>stressed</t>
+        </is>
+      </c>
       <c r="E81" t="n">
-        <v>5.7</v>
+        <v>5.5</v>
       </c>
       <c r="F81" t="n">
         <v>65</v>
       </c>
       <c r="G81" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="H81" t="n">
-        <v>36.52</v>
+        <v>36.43</v>
       </c>
     </row>
     <row r="82">
@@ -2337,25 +2412,25 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>poor sleep</t>
+          <t>sore breasts</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>stressed</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="F82" t="n">
         <v>66</v>
       </c>
       <c r="G82" t="n">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="H82" t="n">
-        <v>36.53</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="83">
@@ -2366,25 +2441,25 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>cravings</t>
+          <t>sore breasts</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>irritable</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="F83" t="n">
         <v>62</v>
       </c>
       <c r="G83" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H83" t="n">
-        <v>36.54</v>
+        <v>36.48</v>
       </c>
     </row>
     <row r="84">
@@ -2395,7 +2470,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>bloating</t>
+          <t>poor sleep</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2404,7 +2479,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>5.4</v>
+        <v>6.2</v>
       </c>
       <c r="F84" t="n">
         <v>63</v>
@@ -2413,7 +2488,7 @@
         <v>49</v>
       </c>
       <c r="H84" t="n">
-        <v>36.28</v>
+        <v>36.26</v>
       </c>
     </row>
     <row r="85">
@@ -2422,14 +2497,24 @@
           <t>2026-03-25</t>
         </is>
       </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>headache</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E85" t="n">
-        <v>6.4</v>
+        <v>6.7</v>
       </c>
       <c r="F85" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G85" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H85" t="n">
         <v>36.28</v>
@@ -2446,22 +2531,27 @@
           <t>heavy</t>
         </is>
       </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>headache</t>
+        </is>
+      </c>
       <c r="D86" t="inlineStr">
         <is>
           <t>okay</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>7.5</v>
+        <v>7.1</v>
       </c>
       <c r="F86" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="G86" t="n">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="H86" t="n">
-        <v>36.21</v>
+        <v>36.23</v>
       </c>
     </row>
     <row r="87">
@@ -2475,27 +2565,22 @@
           <t>heavy</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>backache; low energy</t>
-        </is>
-      </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="F87" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G87" t="n">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="H87" t="n">
-        <v>36.15</v>
+        <v>36.21</v>
       </c>
     </row>
     <row r="88">
@@ -2515,16 +2600,16 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>7.2</v>
+        <v>6.7</v>
       </c>
       <c r="F88" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G88" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H88" t="n">
-        <v>36.11</v>
+        <v>36.05</v>
       </c>
     </row>
     <row r="89">
@@ -2540,20 +2625,20 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E89" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="F89" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="G89" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="H89" t="n">
-        <v>36.23</v>
+        <v>36.15</v>
       </c>
     </row>
     <row r="90">
@@ -2567,22 +2652,27 @@
           <t>spotting</t>
         </is>
       </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>low energy</t>
+        </is>
+      </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>6.8</v>
+        <v>7.9</v>
       </c>
       <c r="F90" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G90" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H90" t="n">
-        <v>36.21</v>
+        <v>36.16</v>
       </c>
     </row>
     <row r="91">
@@ -2592,16 +2682,16 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>6.7</v>
+        <v>7.1</v>
       </c>
       <c r="F91" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G91" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="H91" t="n">
-        <v>36.05</v>
+        <v>36.11</v>
       </c>
     </row>
     <row r="92">
@@ -2610,22 +2700,17 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>great</t>
-        </is>
-      </c>
       <c r="E92" t="n">
-        <v>7.2</v>
+        <v>6.7</v>
       </c>
       <c r="F92" t="n">
         <v>58</v>
       </c>
       <c r="G92" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H92" t="n">
-        <v>36.15</v>
+        <v>36.17</v>
       </c>
     </row>
     <row r="93">
@@ -2635,16 +2720,16 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>7.9</v>
+        <v>8.1</v>
       </c>
       <c r="F93" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G93" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="H93" t="n">
-        <v>36.16</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="94">
@@ -2654,16 +2739,16 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>7.1</v>
+        <v>7.9</v>
       </c>
       <c r="F94" t="n">
         <v>56</v>
       </c>
       <c r="G94" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="H94" t="n">
-        <v>36.11</v>
+        <v>36.14</v>
       </c>
     </row>
     <row r="95">
@@ -2673,16 +2758,16 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>6.7</v>
+        <v>6.9</v>
       </c>
       <c r="F95" t="n">
         <v>58</v>
       </c>
       <c r="G95" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="H95" t="n">
-        <v>36.17</v>
+        <v>36.09</v>
       </c>
     </row>
     <row r="96">
@@ -2692,16 +2777,16 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>8.1</v>
+        <v>7</v>
       </c>
       <c r="F96" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G96" t="n">
         <v>66</v>
       </c>
       <c r="H96" t="n">
-        <v>36.18</v>
+        <v>36.17</v>
       </c>
     </row>
     <row r="97">
@@ -2710,17 +2795,22 @@
           <t>2026-04-06</t>
         </is>
       </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>great</t>
+        </is>
+      </c>
       <c r="E97" t="n">
-        <v>7.9</v>
+        <v>7.5</v>
       </c>
       <c r="F97" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G97" t="n">
         <v>71</v>
       </c>
       <c r="H97" t="n">
-        <v>36.14</v>
+        <v>36.1</v>
       </c>
     </row>
     <row r="98">
@@ -2730,16 +2820,16 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>6.9</v>
+        <v>7.5</v>
       </c>
       <c r="F98" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G98" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="H98" t="n">
-        <v>36.1</v>
+        <v>36.17</v>
       </c>
     </row>
     <row r="99">
@@ -2748,17 +2838,27 @@
           <t>2026-04-08</t>
         </is>
       </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>increased libido</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E99" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F99" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G99" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H99" t="n">
-        <v>36.18</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="100">
@@ -2767,17 +2867,27 @@
           <t>2026-04-09</t>
         </is>
       </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>high energy; increased libido</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>great</t>
+        </is>
+      </c>
       <c r="E100" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="F100" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G100" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H100" t="n">
-        <v>36.17</v>
+        <v>36.25</v>
       </c>
     </row>
     <row r="101">
@@ -2786,14 +2896,24 @@
           <t>2026-04-10</t>
         </is>
       </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>high energy; increased libido</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E101" t="n">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="F101" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G101" t="n">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="H101" t="n">
         <v>36.3</v>
@@ -2805,17 +2925,27 @@
           <t>2026-04-11</t>
         </is>
       </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>high energy; increased libido</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E102" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="F102" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G102" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H102" t="n">
-        <v>36.33</v>
+        <v>36.28</v>
       </c>
     </row>
     <row r="103">
@@ -2828,13 +2958,13 @@
         <v>7.6</v>
       </c>
       <c r="F103" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G103" t="n">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H103" t="n">
-        <v>36.4</v>
+        <v>36.51</v>
       </c>
     </row>
     <row r="104">
@@ -2844,16 +2974,16 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="F104" t="n">
         <v>60</v>
       </c>
       <c r="G104" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H104" t="n">
-        <v>36.52</v>
+        <v>36.43</v>
       </c>
     </row>
     <row r="105">
@@ -2862,11 +2992,6 @@
           <t>2026-04-14</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>okay</t>
-        </is>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2886,10 +3011,10 @@
         <v>62</v>
       </c>
       <c r="G106" t="n">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="H106" t="n">
-        <v>36.4</v>
+        <v>36.46</v>
       </c>
     </row>
     <row r="107">
@@ -2898,22 +3023,17 @@
           <t>2026-04-16</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="E107" t="n">
-        <v>8.1</v>
+        <v>7.6</v>
       </c>
       <c r="F107" t="n">
+        <v>58</v>
+      </c>
+      <c r="G107" t="n">
         <v>60</v>
       </c>
-      <c r="G107" t="n">
-        <v>59</v>
-      </c>
       <c r="H107" t="n">
-        <v>36.55</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="108">
@@ -2923,16 +3043,16 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>8.300000000000001</v>
+        <v>7.1</v>
       </c>
       <c r="F108" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G108" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H108" t="n">
-        <v>36.46</v>
+        <v>36.55</v>
       </c>
     </row>
     <row r="109">
@@ -2947,16 +3067,16 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="F109" t="n">
+        <v>61</v>
+      </c>
+      <c r="G109" t="n">
         <v>62</v>
       </c>
-      <c r="G109" t="n">
-        <v>56</v>
-      </c>
       <c r="H109" t="n">
-        <v>36.51</v>
+        <v>36.45</v>
       </c>
     </row>
     <row r="110">
@@ -2966,16 +3086,16 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>7.4</v>
+        <v>7.7</v>
       </c>
       <c r="F110" t="n">
         <v>60</v>
       </c>
       <c r="G110" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="H110" t="n">
-        <v>36.42</v>
+        <v>36.45</v>
       </c>
     </row>
     <row r="111">
@@ -2986,25 +3106,25 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>headache</t>
+          <t>poor sleep</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>7.6</v>
+        <v>7.3</v>
       </c>
       <c r="F111" t="n">
         <v>61</v>
       </c>
       <c r="G111" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H111" t="n">
-        <v>36.44</v>
+        <v>36.46</v>
       </c>
     </row>
     <row r="112">
@@ -3020,20 +3140,20 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>7.9</v>
+        <v>7.6</v>
       </c>
       <c r="F112" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G112" t="n">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="H112" t="n">
-        <v>36.45</v>
+        <v>36.49</v>
       </c>
     </row>
     <row r="113">
@@ -3043,16 +3163,16 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>6.7</v>
+        <v>7.4</v>
       </c>
       <c r="F113" t="n">
         <v>61</v>
       </c>
       <c r="G113" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H113" t="n">
-        <v>36.47</v>
+        <v>36.46</v>
       </c>
     </row>
     <row r="114">
@@ -3063,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>cravings</t>
+          <t>bloating</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3072,16 +3192,16 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="F114" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G114" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H114" t="n">
-        <v>36.3</v>
+        <v>36.26</v>
       </c>
     </row>
     <row r="115">
@@ -3090,17 +3210,22 @@
           <t>2026-04-24</t>
         </is>
       </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
       <c r="E115" t="n">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="F115" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G115" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H115" t="n">
-        <v>36.37</v>
+        <v>36.35</v>
       </c>
     </row>
     <row r="116">
@@ -3116,7 +3241,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>backache</t>
+          <t>low energy</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3125,16 +3250,16 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>7.6</v>
+        <v>7.2</v>
       </c>
       <c r="F116" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G116" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H116" t="n">
-        <v>36.05</v>
+        <v>36.16</v>
       </c>
     </row>
     <row r="117">
@@ -3148,27 +3273,22 @@
           <t>heavy</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>backache; cramps</t>
-        </is>
-      </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E117" t="n">
-        <v>7.5</v>
+        <v>6.9</v>
       </c>
       <c r="F117" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G117" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="H117" t="n">
-        <v>36.1</v>
+        <v>36.09</v>
       </c>
     </row>
     <row r="118">
@@ -3184,25 +3304,25 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>cramps</t>
+          <t>backache</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>7.1</v>
+        <v>7.4</v>
       </c>
       <c r="F118" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G118" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H118" t="n">
-        <v>36.16</v>
+        <v>36.17</v>
       </c>
     </row>
     <row r="119">
@@ -3216,22 +3336,27 @@
           <t>light</t>
         </is>
       </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>low energy</t>
+        </is>
+      </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="F119" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G119" t="n">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="H119" t="n">
-        <v>36.11</v>
+        <v>36.14</v>
       </c>
     </row>
     <row r="120">
@@ -3245,22 +3370,27 @@
           <t>spotting</t>
         </is>
       </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>low energy</t>
+        </is>
+      </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E120" t="n">
-        <v>7.3</v>
+        <v>6.8</v>
       </c>
       <c r="F120" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G120" t="n">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H120" t="n">
-        <v>36.17</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="121">
@@ -3270,16 +3400,16 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
       <c r="F121" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G121" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H121" t="n">
-        <v>36.17</v>
+        <v>36.14</v>
       </c>
     </row>
     <row r="122">
@@ -3289,16 +3419,16 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>7.6</v>
+        <v>7.2</v>
       </c>
       <c r="F122" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G122" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="H122" t="n">
-        <v>36.17</v>
+        <v>36.03</v>
       </c>
     </row>
     <row r="123">
@@ -3307,22 +3437,17 @@
           <t>2026-05-02</t>
         </is>
       </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>great</t>
-        </is>
-      </c>
       <c r="E123" t="n">
-        <v>7.2</v>
+        <v>7.7</v>
       </c>
       <c r="F123" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G123" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="H123" t="n">
-        <v>36.13</v>
+        <v>36.17</v>
       </c>
     </row>
     <row r="124">
@@ -3331,17 +3456,22 @@
           <t>2026-05-03</t>
         </is>
       </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E124" t="n">
         <v>7.3</v>
       </c>
       <c r="F124" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G124" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="H124" t="n">
-        <v>36.09</v>
+        <v>36.14</v>
       </c>
     </row>
     <row r="125">
@@ -3351,16 +3481,16 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="F125" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G125" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="H125" t="n">
-        <v>36.27</v>
+        <v>36.09</v>
       </c>
     </row>
     <row r="126">
@@ -3373,13 +3503,13 @@
         <v>7.5</v>
       </c>
       <c r="F126" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G126" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H126" t="n">
-        <v>36.15</v>
+        <v>36.1</v>
       </c>
     </row>
     <row r="127">
@@ -3388,17 +3518,27 @@
           <t>2026-05-06</t>
         </is>
       </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>high energy; increased libido</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E127" t="n">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="F127" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G127" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="H127" t="n">
-        <v>36.13</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="128">
@@ -3409,7 +3549,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>high energy</t>
+          <t>high energy; increased libido</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -3418,16 +3558,16 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>6.9</v>
+        <v>8</v>
       </c>
       <c r="F128" t="n">
         <v>57</v>
       </c>
       <c r="G128" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H128" t="n">
-        <v>36.16</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="129">
@@ -3443,20 +3583,20 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>great</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E129" t="n">
-        <v>7.7</v>
+        <v>7.5</v>
       </c>
       <c r="F129" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G129" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H129" t="n">
-        <v>36.25</v>
+        <v>36.26</v>
       </c>
     </row>
     <row r="130">
@@ -3465,22 +3605,27 @@
           <t>2026-05-09</t>
         </is>
       </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>increased libido</t>
+        </is>
+      </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>great</t>
         </is>
       </c>
       <c r="E130" t="n">
-        <v>7</v>
+        <v>8.1</v>
       </c>
       <c r="F130" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G130" t="n">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="H130" t="n">
-        <v>36.34</v>
+        <v>36.33</v>
       </c>
     </row>
     <row r="131">
@@ -3490,16 +3635,16 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>7.7</v>
+        <v>7.9</v>
       </c>
       <c r="F131" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G131" t="n">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="H131" t="n">
-        <v>36.4</v>
+        <v>36.35</v>
       </c>
     </row>
     <row r="132">
@@ -3509,16 +3654,16 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>6.7</v>
+        <v>7.7</v>
       </c>
       <c r="F132" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G132" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="H132" t="n">
-        <v>36.42</v>
+        <v>36.46</v>
       </c>
     </row>
     <row r="133">
@@ -3528,16 +3673,16 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>8</v>
+        <v>7.2</v>
       </c>
       <c r="F133" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G133" t="n">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="H133" t="n">
-        <v>36.51</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="134">
@@ -3547,16 +3692,16 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>8.199999999999999</v>
+        <v>7.9</v>
       </c>
       <c r="F134" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G134" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H134" t="n">
-        <v>36.44</v>
+        <v>36.48</v>
       </c>
     </row>
     <row r="135">
@@ -3566,16 +3711,16 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>7.9</v>
+        <v>7.5</v>
       </c>
       <c r="F135" t="n">
         <v>61</v>
       </c>
       <c r="G135" t="n">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="H135" t="n">
-        <v>36.54</v>
+        <v>36.42</v>
       </c>
     </row>
     <row r="136">
@@ -3585,16 +3730,16 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="F136" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G136" t="n">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="H136" t="n">
-        <v>36.36</v>
+        <v>36.47</v>
       </c>
     </row>
     <row r="137">
@@ -3603,22 +3748,17 @@
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="D137" t="inlineStr">
-        <is>
-          <t>okay</t>
-        </is>
-      </c>
       <c r="E137" t="n">
-        <v>7.4</v>
+        <v>7.8</v>
       </c>
       <c r="F137" t="n">
         <v>61</v>
       </c>
       <c r="G137" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="H137" t="n">
-        <v>36.53</v>
+        <v>36.57</v>
       </c>
     </row>
     <row r="138">
@@ -3627,17 +3767,22 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E138" t="n">
-        <v>7.2</v>
+        <v>6.8</v>
       </c>
       <c r="F138" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G138" t="n">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="H138" t="n">
-        <v>36.57</v>
+        <v>36.47</v>
       </c>
     </row>
     <row r="139">
@@ -3646,27 +3791,17 @@
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>bloating</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="E139" t="n">
-        <v>7.8</v>
+        <v>7.6</v>
       </c>
       <c r="F139" t="n">
         <v>62</v>
       </c>
       <c r="G139" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H139" t="n">
-        <v>36.48</v>
+        <v>36.46</v>
       </c>
     </row>
     <row r="140">
@@ -3675,27 +3810,22 @@
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>cravings</t>
-        </is>
-      </c>
       <c r="D140" t="inlineStr">
         <is>
           <t>okay</t>
         </is>
       </c>
       <c r="E140" t="n">
-        <v>7.6</v>
+        <v>7</v>
       </c>
       <c r="F140" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G140" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="H140" t="n">
-        <v>36.46</v>
+        <v>36.48</v>
       </c>
     </row>
     <row r="141">
@@ -3704,27 +3834,22 @@
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>bloating</t>
-        </is>
-      </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E141" t="n">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="F141" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G141" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H141" t="n">
-        <v>36.55</v>
+        <v>36.54</v>
       </c>
     </row>
     <row r="142">
@@ -3735,7 +3860,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>poor sleep</t>
+          <t>headache</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -3747,13 +3872,13 @@
         <v>6.8</v>
       </c>
       <c r="F142" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G142" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="H142" t="n">
-        <v>36.27</v>
+        <v>36.36</v>
       </c>
     </row>
     <row r="143">
@@ -3764,17 +3889,17 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>irritable</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E143" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="F143" t="n">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G143" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H143" t="n">
         <v>36.28</v>
@@ -3797,16 +3922,16 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>7.8</v>
+        <v>6.9</v>
       </c>
       <c r="F144" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G144" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H144" t="n">
-        <v>36.16</v>
+        <v>36.25</v>
       </c>
     </row>
     <row r="145">
@@ -3822,25 +3947,25 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>backache; headache</t>
+          <t>cramps</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E145" t="n">
-        <v>7.1</v>
+        <v>8</v>
       </c>
       <c r="F145" t="n">
         <v>56</v>
       </c>
       <c r="G145" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H145" t="n">
-        <v>36.02</v>
+        <v>36.06</v>
       </c>
     </row>
     <row r="146">
@@ -3856,20 +3981,20 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>7.2</v>
+        <v>6.7</v>
       </c>
       <c r="F146" t="n">
         <v>57</v>
       </c>
       <c r="G146" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H146" t="n">
-        <v>36.14</v>
+        <v>36.21</v>
       </c>
     </row>
     <row r="147">
@@ -3883,27 +4008,22 @@
           <t>light</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>low energy</t>
-        </is>
-      </c>
       <c r="D147" t="inlineStr">
         <is>
           <t>okay</t>
         </is>
       </c>
       <c r="E147" t="n">
-        <v>7.7</v>
+        <v>7.4</v>
       </c>
       <c r="F147" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G147" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H147" t="n">
-        <v>36.1</v>
+        <v>36.23</v>
       </c>
     </row>
     <row r="148">
@@ -3917,27 +4037,22 @@
           <t>spotting</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>low energy</t>
-        </is>
-      </c>
       <c r="D148" t="inlineStr">
         <is>
           <t>okay</t>
         </is>
       </c>
       <c r="E148" t="n">
-        <v>7.7</v>
+        <v>7.3</v>
       </c>
       <c r="F148" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G148" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H148" t="n">
-        <v>36.22</v>
+        <v>36.19</v>
       </c>
     </row>
     <row r="149">
@@ -3947,16 +4062,16 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>6.6</v>
+        <v>7.6</v>
       </c>
       <c r="F149" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G149" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H149" t="n">
-        <v>36.11</v>
+        <v>36.15</v>
       </c>
     </row>
     <row r="150">
@@ -3966,16 +4081,16 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>7.1</v>
+        <v>7.4</v>
       </c>
       <c r="F150" t="n">
         <v>57</v>
       </c>
       <c r="G150" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H150" t="n">
-        <v>36.21</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="151">
@@ -3984,11 +4099,6 @@
           <t>2026-05-30</t>
         </is>
       </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -3997,16 +4107,16 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>6.8</v>
+        <v>7.4</v>
       </c>
       <c r="F152" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G152" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="H152" t="n">
-        <v>36.1</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="153">
@@ -4015,22 +4125,17 @@
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="E153" t="n">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
       <c r="F153" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G153" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H153" t="n">
-        <v>36.18</v>
+        <v>36.12</v>
       </c>
     </row>
     <row r="154">
@@ -4041,20 +4146,20 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E154" t="n">
         <v>7.6</v>
       </c>
       <c r="F154" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G154" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="H154" t="n">
-        <v>36.17</v>
+        <v>36.18</v>
       </c>
     </row>
     <row r="155">
@@ -4063,17 +4168,22 @@
           <t>2026-06-03</t>
         </is>
       </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E155" t="n">
-        <v>7.1</v>
+        <v>6.9</v>
       </c>
       <c r="F155" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="G155" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="H155" t="n">
-        <v>36.05</v>
+        <v>36.04</v>
       </c>
     </row>
     <row r="156">
@@ -4082,17 +4192,22 @@
           <t>2026-06-04</t>
         </is>
       </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E156" t="n">
-        <v>7.6</v>
+        <v>7.3</v>
       </c>
       <c r="F156" t="n">
         <v>57</v>
       </c>
       <c r="G156" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H156" t="n">
-        <v>36.18</v>
+        <v>36.22</v>
       </c>
     </row>
     <row r="157">
@@ -4101,22 +4216,27 @@
           <t>2026-06-05</t>
         </is>
       </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>high energy</t>
+        </is>
+      </c>
       <c r="D157" t="inlineStr">
         <is>
           <t>great</t>
         </is>
       </c>
       <c r="E157" t="n">
-        <v>7.2</v>
+        <v>7.9</v>
       </c>
       <c r="F157" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G157" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="H157" t="n">
-        <v>36.23</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="158">
@@ -4125,17 +4245,27 @@
           <t>2026-06-06</t>
         </is>
       </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>high energy</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>great</t>
+        </is>
+      </c>
       <c r="E158" t="n">
-        <v>7.3</v>
+        <v>7.4</v>
       </c>
       <c r="F158" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G158" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H158" t="n">
-        <v>36.28</v>
+        <v>36.34</v>
       </c>
     </row>
     <row r="159">
@@ -4144,17 +4274,27 @@
           <t>2026-06-07</t>
         </is>
       </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>increased libido</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E159" t="n">
-        <v>7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F159" t="n">
         <v>57</v>
       </c>
       <c r="G159" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H159" t="n">
-        <v>36.35</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="160">
@@ -4164,16 +4304,16 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>6</v>
+        <v>7.8</v>
       </c>
       <c r="F160" t="n">
         <v>62</v>
       </c>
       <c r="G160" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="H160" t="n">
-        <v>36.46</v>
+        <v>36.48</v>
       </c>
     </row>
     <row r="161">
@@ -4186,13 +4326,13 @@
         <v>7.3</v>
       </c>
       <c r="F161" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G161" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="H161" t="n">
-        <v>36.53</v>
+        <v>36.47</v>
       </c>
     </row>
     <row r="162">
@@ -4201,11 +4341,6 @@
           <t>2026-06-10</t>
         </is>
       </c>
-      <c r="D162" t="inlineStr">
-        <is>
-          <t>okay</t>
-        </is>
-      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -4214,16 +4349,16 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F163" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G163" t="n">
         <v>60</v>
       </c>
       <c r="H163" t="n">
-        <v>36.48</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="164">
@@ -4232,17 +4367,22 @@
           <t>2026-06-12</t>
         </is>
       </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
       <c r="E164" t="n">
-        <v>6.8</v>
+        <v>7.4</v>
       </c>
       <c r="F164" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G164" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="H164" t="n">
-        <v>36.47</v>
+        <v>36.55</v>
       </c>
     </row>
     <row r="165">
@@ -4252,16 +4392,16 @@
         </is>
       </c>
       <c r="E165" t="n">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
       <c r="F165" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G165" t="n">
         <v>59</v>
       </c>
       <c r="H165" t="n">
-        <v>36.47</v>
+        <v>36.48</v>
       </c>
     </row>
     <row r="166">
@@ -4271,16 +4411,16 @@
         </is>
       </c>
       <c r="E166" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="F166" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="G166" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H166" t="n">
-        <v>36.48</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="167">
@@ -4290,13 +4430,13 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>7.3</v>
+        <v>7.4</v>
       </c>
       <c r="F167" t="n">
         <v>61</v>
       </c>
       <c r="G167" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="H167" t="n">
         <v>36.46</v>
@@ -4310,25 +4450,25 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>headache</t>
+          <t>sore breasts</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E168" t="n">
-        <v>7.7</v>
+        <v>7.5</v>
       </c>
       <c r="F168" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G168" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H168" t="n">
-        <v>36.56</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="169">
@@ -4337,17 +4477,27 @@
           <t>2026-06-17</t>
         </is>
       </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>sore breasts</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E169" t="n">
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="F169" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G169" t="n">
         <v>57</v>
       </c>
       <c r="H169" t="n">
-        <v>36.46</v>
+        <v>36.48</v>
       </c>
     </row>
     <row r="170">
@@ -4363,20 +4513,20 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>irritable</t>
         </is>
       </c>
       <c r="E170" t="n">
-        <v>6.7</v>
+        <v>7.2</v>
       </c>
       <c r="F170" t="n">
         <v>61</v>
       </c>
       <c r="G170" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="H170" t="n">
-        <v>36.58</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="171">
@@ -4385,27 +4535,17 @@
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>bloating</t>
-        </is>
-      </c>
-      <c r="D171" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
       <c r="E171" t="n">
-        <v>7.1</v>
+        <v>6.5</v>
       </c>
       <c r="F171" t="n">
         <v>64</v>
       </c>
       <c r="G171" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="H171" t="n">
-        <v>36.27</v>
+        <v>36.36</v>
       </c>
     </row>
     <row r="172">
@@ -4416,25 +4556,25 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>poor sleep</t>
+          <t>bloating</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>irritable</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E172" t="n">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="F172" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G172" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="H172" t="n">
-        <v>36.39</v>
+        <v>36.32</v>
       </c>
     </row>
     <row r="173">
@@ -4448,27 +4588,22 @@
           <t>heavy</t>
         </is>
       </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>headache</t>
-        </is>
-      </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E173" t="n">
-        <v>7.7</v>
+        <v>7.5</v>
       </c>
       <c r="F173" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G173" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="H173" t="n">
-        <v>36.26</v>
+        <v>36.21</v>
       </c>
     </row>
     <row r="174">
@@ -4482,27 +4617,22 @@
           <t>heavy</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>low energy; backache</t>
-        </is>
-      </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E174" t="n">
         <v>7.6</v>
       </c>
       <c r="F174" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G174" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H174" t="n">
-        <v>36.2</v>
+        <v>36.15</v>
       </c>
     </row>
     <row r="175">
@@ -4516,27 +4646,22 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>cramps</t>
-        </is>
-      </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E175" t="n">
-        <v>8.300000000000001</v>
+        <v>7.7</v>
       </c>
       <c r="F175" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G175" t="n">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="H175" t="n">
-        <v>36.19</v>
+        <v>36.16</v>
       </c>
     </row>
     <row r="176">
@@ -4556,16 +4681,16 @@
         </is>
       </c>
       <c r="E176" t="n">
-        <v>7</v>
+        <v>7.8</v>
       </c>
       <c r="F176" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G176" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="H176" t="n">
-        <v>36.21</v>
+        <v>36.09</v>
       </c>
     </row>
     <row r="177">
@@ -4579,27 +4704,22 @@
           <t>spotting</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>low energy</t>
-        </is>
-      </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>okay</t>
         </is>
       </c>
       <c r="E177" t="n">
-        <v>7.1</v>
+        <v>7.4</v>
       </c>
       <c r="F177" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G177" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="H177" t="n">
-        <v>36.14</v>
+        <v>36.13</v>
       </c>
     </row>
     <row r="178">
@@ -4608,17 +4728,22 @@
           <t>2026-06-26</t>
         </is>
       </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E178" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="F178" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G178" t="n">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="H178" t="n">
-        <v>36.18</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="179">
@@ -4627,17 +4752,22 @@
           <t>2026-06-27</t>
         </is>
       </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="E179" t="n">
-        <v>7.5</v>
+        <v>7.2</v>
       </c>
       <c r="F179" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G179" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="H179" t="n">
-        <v>36.18</v>
+        <v>36.16</v>
       </c>
     </row>
     <row r="180">
@@ -4647,16 +4777,16 @@
         </is>
       </c>
       <c r="E180" t="n">
-        <v>6.9</v>
+        <v>7.4</v>
       </c>
       <c r="F180" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G180" t="n">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="H180" t="n">
-        <v>36.17</v>
+        <v>36.25</v>
       </c>
     </row>
     <row r="181">
@@ -4666,16 +4796,16 @@
         </is>
       </c>
       <c r="E181" t="n">
-        <v>8.1</v>
+        <v>7.9</v>
       </c>
       <c r="F181" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G181" t="n">
         <v>67</v>
       </c>
       <c r="H181" t="n">
-        <v>36.17</v>
+        <v>36.16</v>
       </c>
     </row>
     <row r="182">
@@ -4690,16 +4820,16 @@
         </is>
       </c>
       <c r="E182" t="n">
-        <v>7.3</v>
+        <v>6.6</v>
       </c>
       <c r="F182" t="n">
         <v>59</v>
       </c>
       <c r="G182" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H182" t="n">
-        <v>36.12</v>
+        <v>36.16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>